<commit_message>
Rename Requirements.txt to requirements.txt
</commit_message>
<xml_diff>
--- a/Schedule/Sample Data/schedule.xlsx
+++ b/Schedule/Sample Data/schedule.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dell-my.sharepoint.com/personal/jaga_karunanithi_dellteam_com1/Documents/Solvedesktop/solvedesktop/Schedule/Sample Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="11_F25DC773A252ABDACC104882691943CC5ADE58FF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{115504F2-C822-4C2F-826F-9C5BFB8A8129}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="11_F25DC773A252ABDACC104882691943CC5ADE58FF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D0E2CA23-4EA0-4F78-ACFD-74F152C0250F}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="7230" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,25 +33,25 @@
     <t>name</t>
   </si>
   <si>
-    <t>nickname</t>
-  </si>
-  <si>
     <t>918870092425</t>
   </si>
   <si>
     <t>Jagasabarivel</t>
   </si>
   <si>
-    <t>Jaga</t>
-  </si>
-  <si>
     <t>919865975793</t>
   </si>
   <si>
     <t>Shwetha</t>
   </si>
   <si>
-    <t>Shwe</t>
+    <t>charge</t>
+  </si>
+  <si>
+    <t>80</t>
+  </si>
+  <si>
+    <t>40</t>
   </si>
 </sst>
 </file>
@@ -400,26 +400,26 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="C2" s="2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="2" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>8</v>

</xml_diff>